<commit_message>
Push latest changes, including the initial readm.md
</commit_message>
<xml_diff>
--- a/exports/kurt_price_model.xlsx
+++ b/exports/kurt_price_model.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,107 +435,697 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9111.219948399816</v>
+        <v>10851.33352222538</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Year: 1970s</t>
+          <t>new to odometer to bins to 0.0-10000.0</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-1566.269044664477</v>
+        <v>1188.34280997986</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Year: 1980s</t>
+          <t>new to odometer to bins to 10000.0-20000.0</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-1089.028248001507</v>
+        <v>4948.326708857201</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Year: 1990s</t>
+          <t>new to odometer to bins to 100000.0-110000.0</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-1734.708509044422</v>
+        <v>757.775968891509</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Year: 2000s</t>
+          <t>new to odometer to bins to 110000.0-120000.0</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-237.3985317258473</v>
+        <v>540.7953374227732</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Year: 2010s</t>
+          <t>new to odometer to bins to 120000.0-130000.0</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4627.404333548753</v>
+        <v>-84.96700101882594</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Odometer: 0–50k miles</t>
+          <t>new to odometer to bins to 130000.0-140000.0</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4391.092181499475</v>
+        <v>-295.2434126376573</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Odometer: 100–150k miles</t>
+          <t>new to odometer to bins to 140000.0-150000.0</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-1142.591765227797</v>
+        <v>-658.9838245234204</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Odometer: 150–200k miles</t>
+          <t>new to odometer to bins to 150000.0-160000.0</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-2161.109152610105</v>
+        <v>-940.400638235521</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Odometer: 200k miles+</t>
+          <t>new to odometer to bins to 160000.0-170000.0</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-2373.552918866455</v>
+        <v>-1024.243500385193</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Odometer: 50–100k miles</t>
+          <t>new to odometer to bins to 170000.0-180000.0</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1286.161655180612</v>
+        <v>-1433.389849536633</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 180000.0-190000.0</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>-1721.344598020205</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 190000.0-200000.0</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-1918.737056616162</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 20000.0-30000.0</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>5015.48663452963</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 200000.0-210000.0</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-2225.48703996809</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 210000.0-220000.0</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>-2141.194051500243</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 220000.0-230000.0</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>-2330.645315542712</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 230000.0-240000.0</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>-2329.805627391022</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 240000.0-250000.0</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>-2700.353181010933</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 250000.0-260000.0</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>-2934.3068132374</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 260000.0-270000.0</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>-2469.335550273979</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 270000.0-280000.0</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>-2750.045019469671</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 280000.0-290000.0</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>-3340.667932178259</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 290000.0-300000.0</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>-2776.170917978955</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 30000.0-40000.0</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>4584.352217780901</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 40000.0-50000.0</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>4303.982929501899</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 50000.0-60000.0</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>3534.158460112679</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 60000.0-70000.0</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>3093.963957732894</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 70000.0-80000.0</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2673.293362851277</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 80000.0-90000.0</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1900.832418155677</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>new to odometer to bins to 90000.0-100000.0</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1534.010523731098</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>new to year to bins to 1980.0-1985.0</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>-2560.481646819302</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>new to year to bins to 1985.0-1990.0</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>-1737.402878400078</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>new to year to bins to 1990.0-1995.0</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>-2079.823778316492</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>new to year to bins to 1995.0-2000.0</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>-2443.860247181097</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>new to year to bins to 2000.0-2005.0</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>-1705.422015865025</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>new to year to bins to 2005.0-2010.0</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>142.2879528942425</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>new to year to bins to 2010.0-2015.0</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>3704.962958729807</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>new to year to bins to 2015.0-2020.0</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>6679.739654893877</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>collapsed to type to car</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>-1481.814671752875</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>collapsed to type to other to missing</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>-798.2036799712976</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>collapsed to type to suv to crossover</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>-287.32828588781</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>collapsed to type to truck miles</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2495.921228180998</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>collapsed to type to van</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>71.42540941155994</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>collapsed to cylinders to 4 cylinders</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>-1608.240151854249</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>collapsed to cylinders to 6 cylinders</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>-181.1594800670357</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>collapsed to cylinders to 8 cylinders</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1483.109857234654</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>collapsed to cylinders to missing</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>306.2897746881234</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>drive to 4wd</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1276.331944837224</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>drive to fwd</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>-1268.564979226519</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>drive to missing</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>-867.6528940537901</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>drive to rwd</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>859.8859285001831</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>transmission to automatic</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>-1093.818220941686</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>transmission to manual</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>-275.2042329867284</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>transmission to other</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1369.022453908911</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>fuel to diesel</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>3879.129827163426</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>fuel to electric</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>-4065.385182620263</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>fuel to gas</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>-385.5411979881434</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>fuel to hybrid</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>-49.848708316726</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>fuel to other</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>621.6452618147632</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>geo to regions to alask milesa</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1550.224811142963</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>geo to regions to hawaii</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>519.1085630962338</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>geo to regions to midwest</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>-718.4528098943754</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>geo to regions to northeast</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>-1104.763511966562</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>geo to regions to southeast</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>-211.9352785260365</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>geo to regions to west</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>-34.18177383750746</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>manufacturer to tier to economy</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>-754.2282327756503</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>manufacturer to tier to exotic</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>759.3829355456172</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>manufacturer to tier to luxury</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>894.1469541294155</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>manufacturer to tier to mid-mark mileset</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>-899.3016568430255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cleaning things up to ensure they run clean, removing old files.
</commit_message>
<xml_diff>
--- a/exports/kurt_price_model.xlsx
+++ b/exports/kurt_price_model.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B71"/>
+  <dimension ref="A1:B73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,7 +435,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10851.33352222538</v>
+        <v>11783.07498423452</v>
       </c>
     </row>
     <row r="3">
@@ -445,7 +445,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1188.34280997986</v>
+        <v>1993.785713187769</v>
       </c>
     </row>
     <row r="4">
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4948.326708857201</v>
+        <v>4692.002820113515</v>
       </c>
     </row>
     <row r="5">
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>757.775968891509</v>
+        <v>844.0586738760046</v>
       </c>
     </row>
     <row r="6">
@@ -475,7 +475,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>540.7953374227732</v>
+        <v>590.0032952131868</v>
       </c>
     </row>
     <row r="7">
@@ -485,7 +485,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-84.96700101882594</v>
+        <v>-36.04068196651608</v>
       </c>
     </row>
     <row r="8">
@@ -495,7 +495,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-295.2434126376573</v>
+        <v>-193.1732795791414</v>
       </c>
     </row>
     <row r="9">
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-658.9838245234204</v>
+        <v>-563.8464759541235</v>
       </c>
     </row>
     <row r="10">
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-940.400638235521</v>
+        <v>-882.1651313647568</v>
       </c>
     </row>
     <row r="11">
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-1024.243500385193</v>
+        <v>-964.9778561049208</v>
       </c>
     </row>
     <row r="12">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-1433.389849536633</v>
+        <v>-1350.077310440778</v>
       </c>
     </row>
     <row r="13">
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-1721.344598020205</v>
+        <v>-1610.634072481749</v>
       </c>
     </row>
     <row r="14">
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-1918.737056616162</v>
+        <v>-1846.598399044991</v>
       </c>
     </row>
     <row r="15">
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5015.48663452963</v>
+        <v>4810.875639135168</v>
       </c>
     </row>
     <row r="16">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-2225.48703996809</v>
+        <v>-2127.967223440522</v>
       </c>
     </row>
     <row r="17">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-2141.194051500243</v>
+        <v>-1959.641492636541</v>
       </c>
     </row>
     <row r="18">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-2330.645315542712</v>
+        <v>-2328.037244225277</v>
       </c>
     </row>
     <row r="19">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-2329.805627391022</v>
+        <v>-2222.100667643237</v>
       </c>
     </row>
     <row r="20">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-2700.353181010933</v>
+        <v>-2589.790535012691</v>
       </c>
     </row>
     <row r="21">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-2934.3068132374</v>
+        <v>-2756.96449936349</v>
       </c>
     </row>
     <row r="22">
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-2469.335550273979</v>
+        <v>-2338.954779768992</v>
       </c>
     </row>
     <row r="23">
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-2750.045019469671</v>
+        <v>-2727.677563312609</v>
       </c>
     </row>
     <row r="24">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-3340.667932178259</v>
+        <v>-3036.916265975082</v>
       </c>
     </row>
     <row r="25">
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-2776.170917978955</v>
+        <v>-2727.261881335214</v>
       </c>
     </row>
     <row r="26">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4584.352217780901</v>
+        <v>4605.54122178635</v>
       </c>
     </row>
     <row r="27">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4303.982929501899</v>
+        <v>4246.778236433041</v>
       </c>
     </row>
     <row r="28">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3534.158460112679</v>
+        <v>3594.811374372028</v>
       </c>
     </row>
     <row r="29">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>3093.963957732894</v>
+        <v>3143.732316284835</v>
       </c>
     </row>
     <row r="30">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2673.293362851277</v>
+        <v>2704.471915409832</v>
       </c>
     </row>
     <row r="31">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1900.832418155677</v>
+        <v>2025.371261603893</v>
       </c>
     </row>
     <row r="32">
@@ -735,397 +735,417 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1534.010523731098</v>
+        <v>1566.875583187667</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>new to year to bins to 1980.0-1985.0</t>
+          <t>new to odometer to bins to nan</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>-2560.481646819302</v>
+        <v>-2555.482690943011</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>new to year to bins to 1985.0-1990.0</t>
+          <t>new to year to bins to 1980.0-1985.0</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>-1737.402878400078</v>
+        <v>-3425.684761008006</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>new to year to bins to 1990.0-1995.0</t>
+          <t>new to year to bins to 1985.0-1990.0</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>-2079.823778316492</v>
+        <v>-2739.921686791092</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>new to year to bins to 1995.0-2000.0</t>
+          <t>new to year to bins to 1990.0-1995.0</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>-2443.860247181097</v>
+        <v>-3203.258478470698</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>new to year to bins to 2000.0-2005.0</t>
+          <t>new to year to bins to 1995.0-2000.0</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>-1705.422015865025</v>
+        <v>-3369.001213859579</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>new to year to bins to 2005.0-2010.0</t>
+          <t>new to year to bins to 2000.0-2005.0</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>142.2879528942425</v>
+        <v>-2681.697229154209</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>new to year to bins to 2010.0-2015.0</t>
+          <t>new to year to bins to 2005.0-2010.0</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3704.962958729807</v>
+        <v>-810.8143416602638</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>new to year to bins to 2015.0-2020.0</t>
+          <t>new to year to bins to 2010.0-2015.0</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>6679.739654893877</v>
+        <v>2757.936145435612</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>collapsed to type to car</t>
+          <t>new to year to bins to 2015.0-2020.0</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>-1481.814671752875</v>
+        <v>5730.639199004304</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>collapsed to type to other to missing</t>
+          <t>new to year to bins to nan</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>-798.2036799712976</v>
+        <v>7741.802366519305</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>collapsed to type to suv to crossover</t>
+          <t>collapsed to type to car</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>-287.32828588781</v>
+        <v>-1441.637766599376</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>collapsed to type to truck miles</t>
+          <t>collapsed to type to other to missing</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2495.921228180998</v>
+        <v>-805.6704097676812</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>collapsed to type to van</t>
+          <t>collapsed to type to suv to crossover</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>71.42540941155994</v>
+        <v>-261.1474105322304</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>collapsed to cylinders to 4 cylinders</t>
+          <t>collapsed to type to truck miles</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>-1608.240151854249</v>
+        <v>2457.014404295858</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>collapsed to cylinders to 6 cylinders</t>
+          <t>collapsed to type to van</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>-181.1594800670357</v>
+        <v>51.44118261584813</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>collapsed to cylinders to 8 cylinders</t>
+          <t>collapsed to cylinders to 4 cylinders</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1483.109857234654</v>
+        <v>-1604.934613520125</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>collapsed to cylinders to missing</t>
+          <t>collapsed to cylinders to 6 cylinders</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>306.2897746881234</v>
+        <v>-191.3332882702911</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>drive to 4wd</t>
+          <t>collapsed to cylinders to 8 cylinders</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1276.331944837224</v>
+        <v>1478.19206834339</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>drive to fwd</t>
+          <t>collapsed to cylinders to missing</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>-1268.564979226519</v>
+        <v>318.0758334339322</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>drive to missing</t>
+          <t>drive to 4wd</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>-867.6528940537901</v>
+        <v>1273.444497138164</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>drive to rwd</t>
+          <t>drive to fwd</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>859.8859285001831</v>
+        <v>-1229.846625081634</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>transmission to automatic</t>
+          <t>drive to missing</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>-1093.818220941686</v>
+        <v>-896.6728342865375</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>transmission to manual</t>
+          <t>drive to rwd</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>-275.2042329867284</v>
+        <v>853.0749621992215</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>transmission to other</t>
+          <t>transmission to automatic</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1369.022453908911</v>
+        <v>-1134.546168145105</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>fuel to diesel</t>
+          <t>transmission to manual</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>3879.129827163426</v>
+        <v>-271.2586465001261</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>fuel to electric</t>
+          <t>transmission to other</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>-4065.385182620263</v>
+        <v>1405.804814607236</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>fuel to gas</t>
+          <t>fuel to diesel</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>-385.5411979881434</v>
+        <v>3859.450385385093</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>fuel to hybrid</t>
+          <t>fuel to electric</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>-49.848708316726</v>
+        <v>-3790.583312354053</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>fuel to other</t>
+          <t>fuel to gas</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>621.6452618147632</v>
+        <v>-437.7630290626837</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>geo to regions to alask milesa</t>
+          <t>fuel to hybrid</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1550.224811142963</v>
+        <v>-150.2730622182293</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>geo to regions to hawaii</t>
+          <t>fuel to other</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>519.1085630962338</v>
+        <v>519.1690182312957</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>geo to regions to midwest</t>
+          <t>geo to regions to alask milesa</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>-718.4528098943754</v>
+        <v>1474.512139999187</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>geo to regions to northeast</t>
+          <t>geo to regions to hawaii</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>-1104.763511966562</v>
+        <v>500.8511880565279</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>geo to regions to southeast</t>
+          <t>geo to regions to midwest</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>-211.9352785260365</v>
+        <v>-696.4739361094229</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>geo to regions to west</t>
+          <t>geo to regions to northeast</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>-34.18177383750746</v>
+        <v>-1069.7876339166</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>manufacturer to tier to economy</t>
+          <t>geo to regions to southeast</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>-754.2282327756503</v>
+        <v>-198.7986596458507</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>manufacturer to tier to exotic</t>
+          <t>geo to regions to west</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>759.3829355456172</v>
+        <v>-10.30309838839023</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>manufacturer to tier to luxury</t>
+          <t>manufacturer to tier to economy</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>894.1469541294155</v>
+        <v>-745.5956725306718</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
+          <t>manufacturer to tier to exotic</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>738.4615496795533</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>manufacturer to tier to luxury</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>901.5321678676917</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
           <t>manufacturer to tier to mid-mark mileset</t>
         </is>
       </c>
-      <c r="B71" t="n">
-        <v>-899.3016568430255</v>
+      <c r="B73" t="n">
+        <v>-894.3980450252216</v>
       </c>
     </row>
   </sheetData>

</xml_diff>